<commit_message>
modified:   .gitignore 	modified:   content_db.xlsx 	modified:   content_generator.py 	modified:   email_sender.py 	modified:   excel_manager.py 	new file:   generated_images/post_20260309_215606_eab7ff69.png 	new file:   image_generator.py 	modified:   linkedin_poster.py 	modified:   llm_generator.py 	modified:   main.py
	modified:   scheduler.py
</commit_message>
<xml_diff>
--- a/content_db.xlsx
+++ b/content_db.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,15 +456,20 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>image_path</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>when_to_post</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>posted</t>
         </is>
@@ -501,17 +506,18 @@
 How are you integrating Generative AI into your content workflow, or what's holding you back from exploring its potential?</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>2026-03-06</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -548,17 +554,18 @@
 How do you approach ethical considerations in your own AI initiatives or discussions?</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -600,17 +607,18 @@
 #AI #ArtificialIntelligence #AISkills #FutureofWork #CareerDevelopment #TechSkills #PromptEngineering #MachineLearning #JobSeekers #ProfessionalDevelopment</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -637,20 +645,40 @@
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AI for SMEs: Unlocking Growth Without a Data Science Team
+Think AI is only for tech giants? Think again.
+I hear this all the time: "AI is too expensive, too complex, only for companies with huge tech teams." And honestly, I used to think something similar. But I've been diving deep into this lately, and it's simply not true anymore, especially for small and medium-sized businesses.
+We're past the point where you need a data science PhD to get started. There are incredibly accessible AI tools out there that can genuinely transform your operations. I'm talking about things that boost productivity, make customer service AMAZING, and even help you understand your market better than ever. And the best part? They don't break the bank.
+Just a few examples of what I'm seeing:
+• Automating repetitive tasks
+• Personalizing customer interactions
+• Quick insights from market data
+• Streamlining content creation
+My point is, don't let the hype or the perceived complexity scare you off. AI is becoming an essential part of growth, and it's within reach for EVERYONE, not just Silicon Valley. It's time to stop leaving powerful tools on the table.
+What's one area in your business you think AI could REALLY help?
+#AIFreedom #SMBGrowth #SmallBusinessAI #TechForSMEs #ProductivityHacks #CustomerServiceAI #MarketAnalysis #AIStrategy #NoDataScienceTeam</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>C:\Users\nares\OneDrive\Desktop\Linkedin Automation with API\project\generated_images\post_20260309_222436_f0bd58de.png</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -675,20 +703,39 @@
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5 Common AI Myths That Are Holding Your Business Back
+"AI is too expensive," "AI will take all our jobs"... Time to debunk.
+I hear these fears constantly, and honestly, they're holding too many businesses back. We're letting popular misconceptions about AI stop us from exploring powerful solutions. Let's get REAL about what AI actually means for operations today.
+Here's the honest truth:
+• AI isn't just for tech giants. SMEs are leveraging it daily to automate tasks and gain insights.
+• It's not always a massive, complex overhaul. Accessible, scalable tools exist, integrating without breaking the bank.
+• It won't replace all your human employees. It handles repetitive work, freeing your team for creative, strategic tasks. It's about augmentation, not total replacement.
+• AI isn't some futuristic concept. It’s practical, here now, and increasingly user-friendly.
+Don't let outdated fears keep you from serious efficiency and innovation.
+What common AI myth are YOU still encountering?
+#AIMyths #BusinessAI #AIforBusiness #DigitalTransformation #Innovation #FutureofWork #TechDemystified #AIStrategy</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>C:\Users\nares\OneDrive\Desktop\Linkedin Automation with API\project\generated_images\post_20260310_133517_317b77cb.png</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -714,17 +761,18 @@
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -752,17 +800,18 @@
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -790,17 +839,18 @@
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -828,17 +878,18 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -866,17 +917,18 @@
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -904,17 +956,18 @@
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -942,17 +995,18 @@
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -980,17 +1034,18 @@
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>2026-03-18</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1018,17 +1073,18 @@
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1056,17 +1112,18 @@
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1094,17 +1151,18 @@
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1132,17 +1190,18 @@
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>2026-03-22</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1170,17 +1229,18 @@
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
           <t>2026-03-23</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1208,17 +1268,18 @@
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1246,17 +1307,18 @@
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1284,17 +1346,18 @@
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1322,17 +1385,18 @@
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1360,17 +1424,18 @@
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
           <t>2026-03-28</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1398,17 +1463,18 @@
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
           <t>2026-03-29</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1436,17 +1502,18 @@
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
           <t>2026-03-30</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1474,17 +1541,18 @@
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1512,17 +1580,18 @@
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1550,17 +1619,18 @@
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
           <t>2026-04-02</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1588,17 +1658,18 @@
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
           <t>2026-04-03</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1626,17 +1697,18 @@
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
           <t>2026-04-04</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1675,17 +1747,18 @@
 What's the #1 business objective you hope AI will help you achieve in the next year?</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1722,17 +1795,18 @@
 What's the biggest hurdle your organization faces in building a sustainable AI strategy with clear ROI?</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>2026-03-08</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1759,20 +1833,40 @@
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>The AI Strategy Blueprint: 5 Non-Negotiable Steps
+Feeling overwhelmed by AI? 🤯 Here's a clear, actionable path to developing your company's AI strategy.
+The AI revolution is here. But *navigating* it requires more than just hype; it demands a solid blueprint.
+Many businesses struggle to move beyond experimentation. They need a strategic roadmap.
+Here are 5 non-negotiable steps to build your robust AI strategy:
+• **Define Scope &amp; Vision**: What problems will AI solve? Align with business objectives. 🎯
+• **Assess Data Readiness**: Is your data clean, accessible, and structured for AI? This is crucial.
+• **Talent &amp; Culture Audit**: Identify skill gaps. Foster an AI-ready mindset within your team.
+• **Pilot Program Planning**: Start small. Test use cases with measurable KPIs to prove value.
+• **Scale &amp; Integrate**: Once successful, integrate AI solutions deeply into workflows. Expand strategically. 🚀
+This isn't just about technology; it's about transforming your business model. Are you ready to lead the charge?
+#AIStrategy #ArtificialIntelligence #BusinessStrategy #DigitalTransformation #TechLeadership #Innovation #FutureofWork #AIReadiness #StrategicPlanning #EnterpriseAI</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>C:\Users\nares\OneDrive\Desktop\Linkedin Automation with API\project\generated_images\post_20260309_215636_5c9c6905.png</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1797,18 +1891,37 @@
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Data Is Your AI's Fuel: Is Your Tank Empty?
+An AI model is only as good as the data it's fed. Is your data strategy robust enough?
+I’ve been having a lot of conversations lately, and it's clear many are rushing into AI without first looking under the hood. We invest in shiny new models, powerful platforms, but often neglect the single most IMPORTANT ingredient: our data.
+I’ve seen promising AI initiatives stall, even fail, because the underlying data was a mess. It’s a harsh truth: complex algorithms can't magically fix poor data quality, inconsistent governance, or siloed information. They just amplify existing problems.
+Think of your data as the fuel for your AI. If the tank is full of sludge, your engine won’t run. We need to prioritize making sure our data is:
+• Clean and accurate
+• Governed properly
+• Easily accessible
+This foundational work makes all the difference. Don't just chase the next impressive AI tool. Let's get serious about data readiness first.
+What’s the biggest data challenge you’re tackling right now?
+#DataStrategy #AIReadiness #DataQuality #AIFuel #DataGovernance #AIInitiatives #DataDriven #DigitalTransformation</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>C:\Users\nares\OneDrive\Desktop\Linkedin Automation with API\project\generated_images\post_20260310_133607_f25fe7d7.png</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
           <t>2026-03-10</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1836,17 +1949,18 @@
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1874,17 +1988,18 @@
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
           <t>2026-03-12</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1912,17 +2027,18 @@
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1950,17 +2066,18 @@
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
           <t>2026-03-14</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1988,17 +2105,18 @@
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2026,17 +2144,18 @@
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
           <t>2026-03-16</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2064,17 +2183,18 @@
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2102,17 +2222,18 @@
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
           <t>2026-03-18</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2140,17 +2261,18 @@
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2178,17 +2300,18 @@
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
           <t>2026-03-20</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2216,17 +2339,18 @@
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2254,17 +2378,18 @@
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
           <t>2026-03-22</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2292,17 +2417,18 @@
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
           <t>2026-03-23</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2330,17 +2456,18 @@
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2368,17 +2495,18 @@
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2406,17 +2534,18 @@
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2444,17 +2573,18 @@
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2482,17 +2612,18 @@
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
           <t>2026-03-28</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2520,17 +2651,18 @@
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
           <t>2026-03-29</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2558,17 +2690,18 @@
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
           <t>2026-03-30</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2596,17 +2729,18 @@
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
           <t>2026-03-31</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2634,17 +2768,18 @@
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2672,17 +2807,18 @@
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
           <t>2026-04-02</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2710,17 +2846,18 @@
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
           <t>2026-04-03</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2748,17 +2885,18 @@
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
           <t>2026-04-04</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2786,17 +2924,18 @@
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
           <t>2026-04-05</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>